<commit_message>
10/22 redo TBFxFRI interaction figure
</commit_message>
<xml_diff>
--- a/fire nutrient/raw_data/Nutrient Supply Rate Data Project_2605_first_batch_2025.xlsx
+++ b/fire nutrient/raw_data/Nutrient Supply Rate Data Project_2605_first_batch_2025.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kishari\Documents\Kishari\Clients\Current clients\Allison Louthan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\PhD\VFT\VFT_github\zyao78VFTcode\fire nutrient\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BDAB002-E6B5-4D5C-BF06-4D20750EE1B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16457" windowHeight="5537"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="23236" windowHeight="13875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Shipment_7068" sheetId="1" r:id="rId1"/>
@@ -33,179 +34,180 @@
     <t>Shipment 7068, Received 2025-11-10</t>
   </si>
   <si>
+    <t>WAL #</t>
+  </si>
+  <si>
+    <t>Sample ID</t>
+  </si>
+  <si>
+    <t>Burial Date</t>
+  </si>
+  <si>
+    <t>Retrieval Date</t>
+  </si>
+  <si>
+    <t># Anion</t>
+  </si>
+  <si>
+    <t># Cation</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>Total N</t>
+  </si>
+  <si>
+    <t>NO3-N</t>
+  </si>
+  <si>
+    <t>NH4-N</t>
+  </si>
+  <si>
+    <t>Ca</t>
+  </si>
+  <si>
+    <t>Mg</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>Fe</t>
+  </si>
+  <si>
+    <t>Mn</t>
+  </si>
+  <si>
+    <t>Cu</t>
+  </si>
+  <si>
+    <t>Zn</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>Pb</t>
+  </si>
+  <si>
+    <t>Al</t>
+  </si>
+  <si>
+    <t>Cd</t>
+  </si>
+  <si>
+    <t>Method Detection Limits (mdl):</t>
+  </si>
+  <si>
+    <t>CH #1</t>
+  </si>
+  <si>
+    <t>2025-06-13</t>
+  </si>
+  <si>
+    <t>2025-10-14</t>
+  </si>
+  <si>
+    <t>CH #2</t>
+  </si>
+  <si>
+    <t>CH #3</t>
+  </si>
+  <si>
+    <t>CM #1</t>
+  </si>
+  <si>
+    <t>CM #2</t>
+  </si>
+  <si>
+    <t>CM #3</t>
+  </si>
+  <si>
+    <t>HS Site1 B1</t>
+  </si>
+  <si>
+    <t>2025-06-18</t>
+  </si>
+  <si>
+    <t>2025-10-15</t>
+  </si>
+  <si>
+    <t>HS SIte1 B3</t>
+  </si>
+  <si>
+    <t>HS Site1 B2</t>
+  </si>
+  <si>
+    <t>HS Site1 B4</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> probe burnt</t>
+  </si>
+  <si>
+    <t>HS Site2 B1</t>
+  </si>
+  <si>
+    <t>HS Site2 B2</t>
+  </si>
+  <si>
+    <t>HS Site2 B3</t>
+  </si>
+  <si>
+    <t>HS Site2 B4</t>
+  </si>
+  <si>
+    <t>probe burnt</t>
+  </si>
+  <si>
+    <t>HS Site3 B1</t>
+  </si>
+  <si>
+    <t>HS Site3 B2</t>
+  </si>
+  <si>
+    <t>HS Site3 B3</t>
+  </si>
+  <si>
+    <t>HS Site3 B4</t>
+  </si>
+  <si>
+    <t>GSP-LI #1</t>
+  </si>
+  <si>
+    <t>2025-06-16</t>
+  </si>
+  <si>
+    <t>GSP-LI #2</t>
+  </si>
+  <si>
+    <t>GSP-LI #3</t>
+  </si>
+  <si>
+    <t>GSP-BI #1</t>
+  </si>
+  <si>
+    <t>GSP-BI #2</t>
+  </si>
+  <si>
+    <t>GSP-BI #3</t>
+  </si>
+  <si>
     <t>PRS(tm)-probe supply rate (micro grams/10cm2/burial length)</t>
-  </si>
-  <si>
-    <t>WAL #</t>
-  </si>
-  <si>
-    <t>Sample ID</t>
-  </si>
-  <si>
-    <t>Burial Date</t>
-  </si>
-  <si>
-    <t>Retrieval Date</t>
-  </si>
-  <si>
-    <t># Anion</t>
-  </si>
-  <si>
-    <t># Cation</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Total N</t>
-  </si>
-  <si>
-    <t>NO3-N</t>
-  </si>
-  <si>
-    <t>NH4-N</t>
-  </si>
-  <si>
-    <t>Ca</t>
-  </si>
-  <si>
-    <t>Mg</t>
-  </si>
-  <si>
-    <t>K</t>
-  </si>
-  <si>
-    <t>P</t>
-  </si>
-  <si>
-    <t>Fe</t>
-  </si>
-  <si>
-    <t>Mn</t>
-  </si>
-  <si>
-    <t>Cu</t>
-  </si>
-  <si>
-    <t>Zn</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>Pb</t>
-  </si>
-  <si>
-    <t>Al</t>
-  </si>
-  <si>
-    <t>Cd</t>
-  </si>
-  <si>
-    <t>Method Detection Limits (mdl):</t>
-  </si>
-  <si>
-    <t>CH #1</t>
-  </si>
-  <si>
-    <t>2025-06-13</t>
-  </si>
-  <si>
-    <t>2025-10-14</t>
-  </si>
-  <si>
-    <t>CH #2</t>
-  </si>
-  <si>
-    <t>CH #3</t>
-  </si>
-  <si>
-    <t>CM #1</t>
-  </si>
-  <si>
-    <t>CM #2</t>
-  </si>
-  <si>
-    <t>CM #3</t>
-  </si>
-  <si>
-    <t>HS Site1 B1</t>
-  </si>
-  <si>
-    <t>2025-06-18</t>
-  </si>
-  <si>
-    <t>2025-10-15</t>
-  </si>
-  <si>
-    <t>HS SIte1 B3</t>
-  </si>
-  <si>
-    <t>HS Site1 B2</t>
-  </si>
-  <si>
-    <t>HS Site1 B4</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> probe burnt</t>
-  </si>
-  <si>
-    <t>HS Site2 B1</t>
-  </si>
-  <si>
-    <t>HS Site2 B2</t>
-  </si>
-  <si>
-    <t>HS Site2 B3</t>
-  </si>
-  <si>
-    <t>HS Site2 B4</t>
-  </si>
-  <si>
-    <t>probe burnt</t>
-  </si>
-  <si>
-    <t>HS Site3 B1</t>
-  </si>
-  <si>
-    <t>HS Site3 B2</t>
-  </si>
-  <si>
-    <t>HS Site3 B3</t>
-  </si>
-  <si>
-    <t>HS Site3 B4</t>
-  </si>
-  <si>
-    <t>GSP-LI #1</t>
-  </si>
-  <si>
-    <t>2025-06-16</t>
-  </si>
-  <si>
-    <t>GSP-LI #2</t>
-  </si>
-  <si>
-    <t>GSP-LI #3</t>
-  </si>
-  <si>
-    <t>GSP-BI #1</t>
-  </si>
-  <si>
-    <t>GSP-BI #2</t>
-  </si>
-  <si>
-    <t>GSP-BI #3</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -216,12 +218,20 @@
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="DengXian"/>
+      <family val="3"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="3">
@@ -254,14 +264,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -280,9 +290,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -320,7 +330,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -392,7 +402,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -565,226 +575,226 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z31"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A2" s="4" t="s">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.45">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="6"/>
+      <c r="R1" s="6"/>
+      <c r="S1" s="6"/>
+      <c r="T1" s="6"/>
+      <c r="U1" s="6"/>
+      <c r="V1" s="6"/>
+      <c r="W1" s="6"/>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.45">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
-      <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
-      <c r="I2" s="3"/>
-      <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
-      <c r="N2" s="3"/>
-      <c r="O2" s="3"/>
-      <c r="P2" s="3"/>
-      <c r="Q2" s="3"/>
-      <c r="R2" s="3"/>
-      <c r="S2" s="3"/>
-      <c r="T2" s="3"/>
-      <c r="U2" s="3"/>
-      <c r="V2" s="3"/>
-      <c r="W2" s="3"/>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
-      <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
-      <c r="U3" s="3"/>
-      <c r="V3" s="3"/>
-      <c r="W3" s="3"/>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A4" s="5" t="s">
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
+      <c r="S2" s="6"/>
+      <c r="T2" s="6"/>
+      <c r="U2" s="6"/>
+      <c r="V2" s="6"/>
+      <c r="W2" s="6"/>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.45">
+      <c r="A3" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+      <c r="M3" s="6"/>
+      <c r="N3" s="6"/>
+      <c r="O3" s="6"/>
+      <c r="P3" s="6"/>
+      <c r="Q3" s="6"/>
+      <c r="R3" s="6"/>
+      <c r="S3" s="6"/>
+      <c r="T3" s="6"/>
+      <c r="U3" s="6"/>
+      <c r="V3" s="6"/>
+      <c r="W3" s="6"/>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.45">
+      <c r="A4" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="Q4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="U4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A5" s="5" t="s">
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+      <c r="M4" s="6"/>
+      <c r="N4" s="6"/>
+      <c r="O4" s="6"/>
+      <c r="P4" s="6"/>
+      <c r="Q4" s="6"/>
+      <c r="R4" s="6"/>
+      <c r="S4" s="6"/>
+      <c r="T4" s="6"/>
+      <c r="U4" s="6"/>
+      <c r="V4" s="6"/>
+      <c r="W4" s="6"/>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.45">
+      <c r="A5" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
+      <c r="P5" s="6"/>
+      <c r="Q5" s="6"/>
+      <c r="R5" s="6"/>
+      <c r="S5" s="6"/>
+      <c r="T5" s="6"/>
+      <c r="U5" s="6"/>
+      <c r="V5" s="6"/>
+      <c r="W5" s="6"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.45">
+      <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="Q5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="U5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="s">
+      <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="G6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="1" t="s">
+      <c r="N6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="N6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="P6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="Q6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="Q6" s="1" t="s">
+      <c r="R6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="R6" s="1" t="s">
+      <c r="S6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="S6" s="1" t="s">
+      <c r="T6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="T6" s="1" t="s">
+      <c r="U6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="U6" s="1" t="s">
+      <c r="V6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="V6" s="1" t="s">
+      <c r="W6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="W6" s="1" t="s">
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.45">
+      <c r="A7" s="5" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.4">
-      <c r="A7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
       <c r="H7" s="1">
         <v>2</v>
       </c>
@@ -837,1266 +847,1266 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>254942</v>
       </c>
       <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s">
         <v>29</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>30</v>
       </c>
-      <c r="D8" t="s">
-        <v>31</v>
-      </c>
       <c r="E8">
         <v>2</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="3">
         <v>11.9</v>
       </c>
-      <c r="I8" s="8">
+      <c r="I8" s="4">
         <v>0.6</v>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="3">
         <v>11.3</v>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="3">
         <v>312</v>
       </c>
-      <c r="L8" s="7">
+      <c r="L8" s="3">
         <v>322.10000000000002</v>
       </c>
-      <c r="M8" s="7">
+      <c r="M8" s="3">
         <v>294.10000000000002</v>
       </c>
-      <c r="N8" s="8">
-        <v>0</v>
-      </c>
-      <c r="O8" s="7">
+      <c r="N8" s="4">
+        <v>0</v>
+      </c>
+      <c r="O8" s="3">
         <v>12.62</v>
       </c>
-      <c r="P8" s="7">
+      <c r="P8" s="3">
         <v>1.78</v>
       </c>
-      <c r="Q8" s="7">
+      <c r="Q8" s="3">
         <v>0.436</v>
       </c>
-      <c r="R8" s="7">
+      <c r="R8" s="3">
         <v>0.86</v>
       </c>
-      <c r="S8" s="8">
+      <c r="S8" s="4">
         <v>0.14000000000000001</v>
       </c>
-      <c r="T8" s="7">
+      <c r="T8" s="3">
         <v>120.4</v>
       </c>
-      <c r="U8" s="7">
+      <c r="U8" s="3">
         <v>5.7320000000000002</v>
       </c>
-      <c r="V8" s="7">
+      <c r="V8" s="3">
         <v>17.399999999999999</v>
       </c>
       <c r="W8" s="2">
         <v>0</v>
       </c>
-      <c r="X8" s="7"/>
-    </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="X8" s="3"/>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>254943</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" t="s">
         <v>30</v>
       </c>
-      <c r="D9" t="s">
-        <v>31</v>
-      </c>
       <c r="E9">
         <v>2</v>
       </c>
       <c r="F9">
         <v>2</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="3">
         <v>7.7</v>
       </c>
-      <c r="I9" s="8">
+      <c r="I9" s="4">
         <v>0.4</v>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="3">
         <v>7.3</v>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="3">
         <v>181</v>
       </c>
-      <c r="L9" s="7">
+      <c r="L9" s="3">
         <v>320.89999999999998</v>
       </c>
-      <c r="M9" s="7">
+      <c r="M9" s="3">
         <v>119</v>
       </c>
-      <c r="N9" s="8">
+      <c r="N9" s="4">
         <v>0.11</v>
       </c>
-      <c r="O9" s="7">
+      <c r="O9" s="3">
         <v>828.86</v>
       </c>
-      <c r="P9" s="7">
+      <c r="P9" s="3">
         <v>1.0900000000000001</v>
       </c>
-      <c r="Q9" s="8">
+      <c r="Q9" s="4">
         <v>0.14799999999999999</v>
       </c>
-      <c r="R9" s="7">
+      <c r="R9" s="3">
         <v>7.74</v>
       </c>
-      <c r="S9" s="7">
+      <c r="S9" s="3">
         <v>0.3</v>
       </c>
-      <c r="T9" s="7">
+      <c r="T9" s="3">
         <v>111</v>
       </c>
-      <c r="U9" s="7">
+      <c r="U9" s="3">
         <v>52.341999999999999</v>
       </c>
-      <c r="V9" s="7">
+      <c r="V9" s="3">
         <v>64.900000000000006</v>
       </c>
       <c r="W9" s="2">
         <v>0</v>
       </c>
-      <c r="X9" s="7"/>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="X9" s="3"/>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>254944</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" t="s">
         <v>30</v>
       </c>
-      <c r="D10" t="s">
-        <v>31</v>
-      </c>
       <c r="E10">
         <v>2</v>
       </c>
       <c r="F10">
         <v>2</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="3">
         <v>7.9</v>
       </c>
-      <c r="I10" s="8">
+      <c r="I10" s="4">
         <v>0.7</v>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="3">
         <v>7.2</v>
       </c>
-      <c r="K10" s="7">
+      <c r="K10" s="3">
         <v>222</v>
       </c>
-      <c r="L10" s="7">
+      <c r="L10" s="3">
         <v>287</v>
       </c>
-      <c r="M10" s="7">
+      <c r="M10" s="3">
         <v>246.7</v>
       </c>
-      <c r="N10" s="8">
-        <v>0</v>
-      </c>
-      <c r="O10" s="7">
+      <c r="N10" s="4">
+        <v>0</v>
+      </c>
+      <c r="O10" s="3">
         <v>12.07</v>
       </c>
-      <c r="P10" s="7">
+      <c r="P10" s="3">
         <v>0.88</v>
       </c>
-      <c r="Q10" s="7">
+      <c r="Q10" s="3">
         <v>0.29399999999999998</v>
       </c>
-      <c r="R10" s="7">
+      <c r="R10" s="3">
         <v>0.57999999999999996</v>
       </c>
-      <c r="S10" s="8">
+      <c r="S10" s="4">
         <v>0.13</v>
       </c>
-      <c r="T10" s="7">
+      <c r="T10" s="3">
         <v>122.1</v>
       </c>
-      <c r="U10" s="7">
+      <c r="U10" s="3">
         <v>2.2040000000000002</v>
       </c>
-      <c r="V10" s="7">
+      <c r="V10" s="3">
         <v>25.1</v>
       </c>
       <c r="W10" s="2">
         <v>0</v>
       </c>
-      <c r="X10" s="7"/>
-    </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="X10" s="3"/>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>254945</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" t="s">
         <v>30</v>
       </c>
-      <c r="D11" t="s">
-        <v>31</v>
-      </c>
       <c r="E11">
         <v>2</v>
       </c>
       <c r="F11">
         <v>2</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="3">
         <v>8.1</v>
       </c>
-      <c r="I11" s="8">
+      <c r="I11" s="4">
         <v>0.6</v>
       </c>
-      <c r="J11" s="7">
+      <c r="J11" s="3">
         <v>7.5</v>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="3">
         <v>602</v>
       </c>
-      <c r="L11" s="7">
+      <c r="L11" s="3">
         <v>623.79999999999995</v>
       </c>
-      <c r="M11" s="7">
+      <c r="M11" s="3">
         <v>27.5</v>
       </c>
-      <c r="N11" s="7">
+      <c r="N11" s="3">
         <v>0.7</v>
       </c>
-      <c r="O11" s="7">
+      <c r="O11" s="3">
         <v>102.17</v>
       </c>
-      <c r="P11" s="7">
+      <c r="P11" s="3">
         <v>0.87</v>
       </c>
-      <c r="Q11" s="7">
+      <c r="Q11" s="3">
         <v>0.36599999999999999</v>
       </c>
-      <c r="R11" s="7">
+      <c r="R11" s="3">
         <v>0.64</v>
       </c>
-      <c r="S11" s="7">
+      <c r="S11" s="3">
         <v>0.21</v>
       </c>
-      <c r="T11" s="7">
+      <c r="T11" s="3">
         <v>60.4</v>
       </c>
-      <c r="U11" s="7">
+      <c r="U11" s="3">
         <v>1.5880000000000001</v>
       </c>
-      <c r="V11" s="7">
+      <c r="V11" s="3">
         <v>54.1</v>
       </c>
       <c r="W11" s="2">
         <v>0.05</v>
       </c>
-      <c r="X11" s="7"/>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="X11" s="3"/>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>254946</v>
       </c>
       <c r="B12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" t="s">
         <v>30</v>
       </c>
-      <c r="D12" t="s">
-        <v>31</v>
-      </c>
       <c r="E12">
         <v>2</v>
       </c>
       <c r="F12">
         <v>2</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="3">
         <v>13.2</v>
       </c>
-      <c r="I12" s="8">
+      <c r="I12" s="4">
         <v>0.7</v>
       </c>
-      <c r="J12" s="7">
+      <c r="J12" s="3">
         <v>12.5</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="3">
         <v>181</v>
       </c>
-      <c r="L12" s="7">
+      <c r="L12" s="3">
         <v>431.3</v>
       </c>
-      <c r="M12" s="7">
+      <c r="M12" s="3">
         <v>36.5</v>
       </c>
-      <c r="N12" s="8">
-        <v>0</v>
-      </c>
-      <c r="O12" s="7">
+      <c r="N12" s="4">
+        <v>0</v>
+      </c>
+      <c r="O12" s="3">
         <v>721.29</v>
       </c>
-      <c r="P12" s="7">
+      <c r="P12" s="3">
         <v>0.9</v>
       </c>
-      <c r="Q12" s="7">
+      <c r="Q12" s="3">
         <v>1.8240000000000001</v>
       </c>
-      <c r="R12" s="7">
+      <c r="R12" s="3">
         <v>5.22</v>
       </c>
-      <c r="S12" s="7">
+      <c r="S12" s="3">
         <v>0.39</v>
       </c>
-      <c r="T12" s="7">
+      <c r="T12" s="3">
         <v>38.299999999999997</v>
       </c>
-      <c r="U12" s="7">
+      <c r="U12" s="3">
         <v>1.706</v>
       </c>
-      <c r="V12" s="7">
+      <c r="V12" s="3">
         <v>173.5</v>
       </c>
       <c r="W12" s="2">
         <v>0.03</v>
       </c>
-      <c r="X12" s="7"/>
-    </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="X12" s="3"/>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>254947</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" t="s">
         <v>30</v>
       </c>
-      <c r="D13" t="s">
-        <v>31</v>
-      </c>
       <c r="E13">
         <v>2</v>
       </c>
       <c r="F13">
         <v>2</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="3">
         <v>5</v>
       </c>
-      <c r="I13" s="8">
+      <c r="I13" s="4">
         <v>0.9</v>
       </c>
-      <c r="J13" s="7">
+      <c r="J13" s="3">
         <v>4.0999999999999996</v>
       </c>
-      <c r="K13" s="7">
+      <c r="K13" s="3">
         <v>57</v>
       </c>
-      <c r="L13" s="7">
+      <c r="L13" s="3">
         <v>219.5</v>
       </c>
-      <c r="M13" s="7">
+      <c r="M13" s="3">
         <v>16.399999999999999</v>
       </c>
-      <c r="N13" s="8">
-        <v>0</v>
-      </c>
-      <c r="O13" s="7">
+      <c r="N13" s="4">
+        <v>0</v>
+      </c>
+      <c r="O13" s="3">
         <v>707.02</v>
       </c>
-      <c r="P13" s="7">
+      <c r="P13" s="3">
         <v>1.06</v>
       </c>
-      <c r="Q13" s="8">
+      <c r="Q13" s="4">
         <v>0.16600000000000001</v>
       </c>
-      <c r="R13" s="7">
+      <c r="R13" s="3">
         <v>0.44</v>
       </c>
-      <c r="S13" s="7">
+      <c r="S13" s="3">
         <v>0.31</v>
       </c>
-      <c r="T13" s="7">
+      <c r="T13" s="3">
         <v>194.5</v>
       </c>
-      <c r="U13" s="7">
+      <c r="U13" s="3">
         <v>2.306</v>
       </c>
-      <c r="V13" s="7">
+      <c r="V13" s="3">
         <v>551.70000000000005</v>
       </c>
       <c r="W13">
         <v>0.216</v>
       </c>
-      <c r="X13" s="7"/>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="X13" s="3"/>
+    </row>
+    <row r="14" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>254948</v>
       </c>
       <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" t="s">
         <v>37</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>38</v>
       </c>
-      <c r="D14" t="s">
-        <v>39</v>
-      </c>
       <c r="E14">
         <v>2</v>
       </c>
       <c r="F14">
         <v>2</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="3">
         <v>6</v>
       </c>
-      <c r="I14" s="8">
+      <c r="I14" s="4">
         <v>1.2</v>
       </c>
-      <c r="J14" s="7">
+      <c r="J14" s="3">
         <v>4.8</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="3">
         <v>1670</v>
       </c>
-      <c r="L14" s="7">
+      <c r="L14" s="3">
         <v>513.4</v>
       </c>
-      <c r="M14" s="7">
+      <c r="M14" s="3">
         <v>29.6</v>
       </c>
-      <c r="N14" s="7">
+      <c r="N14" s="3">
         <v>0.56999999999999995</v>
       </c>
-      <c r="O14" s="7">
+      <c r="O14" s="3">
         <v>11.52</v>
       </c>
-      <c r="P14" s="7">
+      <c r="P14" s="3">
         <v>1.1200000000000001</v>
       </c>
-      <c r="Q14" s="7">
+      <c r="Q14" s="3">
         <v>0.20799999999999999</v>
       </c>
-      <c r="R14" s="7">
+      <c r="R14" s="3">
         <v>0.98</v>
       </c>
-      <c r="S14" s="7">
+      <c r="S14" s="3">
         <v>1.2</v>
       </c>
-      <c r="T14" s="7">
+      <c r="T14" s="3">
         <v>379.7</v>
       </c>
-      <c r="U14" s="7">
+      <c r="U14" s="3">
         <v>1.1379999999999999</v>
       </c>
-      <c r="V14" s="7">
+      <c r="V14" s="3">
         <v>42</v>
       </c>
       <c r="W14" s="2">
         <v>0.14799999999999999</v>
       </c>
-      <c r="X14" s="7"/>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="X14" s="3"/>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>254949</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15" t="s">
         <v>38</v>
       </c>
-      <c r="D15" t="s">
-        <v>39</v>
-      </c>
       <c r="E15">
         <v>2</v>
       </c>
       <c r="F15">
         <v>2</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="3">
         <v>6.6</v>
       </c>
-      <c r="I15" s="8">
+      <c r="I15" s="4">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="3">
         <v>5.5</v>
       </c>
-      <c r="K15" s="7">
+      <c r="K15" s="3">
         <v>1380</v>
       </c>
-      <c r="L15" s="7">
+      <c r="L15" s="3">
         <v>428.7</v>
       </c>
-      <c r="M15" s="7">
+      <c r="M15" s="3">
         <v>12.8</v>
       </c>
-      <c r="N15" s="8">
-        <v>0</v>
-      </c>
-      <c r="O15" s="7">
+      <c r="N15" s="4">
+        <v>0</v>
+      </c>
+      <c r="O15" s="3">
         <v>4.9400000000000004</v>
       </c>
-      <c r="P15" s="7">
+      <c r="P15" s="3">
         <v>0.85</v>
       </c>
-      <c r="Q15" s="7">
+      <c r="Q15" s="3">
         <v>0.23599999999999999</v>
       </c>
-      <c r="R15" s="7">
+      <c r="R15" s="3">
         <v>0.24</v>
       </c>
-      <c r="S15" s="8">
-        <v>0</v>
-      </c>
-      <c r="T15" s="7">
+      <c r="S15" s="4">
+        <v>0</v>
+      </c>
+      <c r="T15" s="3">
         <v>266.89999999999998</v>
       </c>
-      <c r="U15" s="7">
+      <c r="U15" s="3">
         <v>1.758</v>
       </c>
-      <c r="V15" s="7">
+      <c r="V15" s="3">
         <v>15.9</v>
       </c>
       <c r="W15" s="2">
         <v>0.13200000000000001</v>
       </c>
-      <c r="X15" s="7"/>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.4">
+      <c r="X15" s="3"/>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>254950</v>
       </c>
       <c r="B16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D16" t="s">
         <v>38</v>
       </c>
-      <c r="D16" t="s">
-        <v>39</v>
-      </c>
       <c r="E16">
         <v>2</v>
       </c>
       <c r="F16">
         <v>2</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="3">
         <v>6.2</v>
       </c>
-      <c r="I16" s="8">
+      <c r="I16" s="4">
         <v>0.9</v>
       </c>
-      <c r="J16" s="7">
+      <c r="J16" s="3">
         <v>5.3</v>
       </c>
-      <c r="K16" s="7">
+      <c r="K16" s="3">
         <v>660</v>
       </c>
-      <c r="L16" s="7">
+      <c r="L16" s="3">
         <v>185.9</v>
       </c>
-      <c r="M16" s="7">
+      <c r="M16" s="3">
         <v>40.299999999999997</v>
       </c>
-      <c r="N16" s="8">
-        <v>0</v>
-      </c>
-      <c r="O16" s="7">
+      <c r="N16" s="4">
+        <v>0</v>
+      </c>
+      <c r="O16" s="3">
         <v>10.92</v>
       </c>
-      <c r="P16" s="7">
+      <c r="P16" s="3">
         <v>0.54</v>
       </c>
-      <c r="Q16" s="8">
+      <c r="Q16" s="4">
         <v>0.11</v>
       </c>
-      <c r="R16" s="7">
+      <c r="R16" s="3">
         <v>0.4</v>
       </c>
-      <c r="S16" s="8">
+      <c r="S16" s="4">
         <v>0.03</v>
       </c>
-      <c r="T16" s="7">
+      <c r="T16" s="3">
         <v>95.5</v>
       </c>
-      <c r="U16" s="7">
+      <c r="U16" s="3">
         <v>0.65900000000000003</v>
       </c>
-      <c r="V16" s="7">
+      <c r="V16" s="3">
         <v>12.6</v>
       </c>
       <c r="W16" s="2">
         <v>0.14899999999999999</v>
       </c>
-      <c r="X16" s="7"/>
-    </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X16" s="3"/>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>254951</v>
       </c>
       <c r="B17" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17">
+        <v>2</v>
+      </c>
+      <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="G17" t="s">
         <v>42</v>
       </c>
-      <c r="C17" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" t="s">
-        <v>39</v>
-      </c>
-      <c r="E17">
-        <v>2</v>
-      </c>
-      <c r="F17">
-        <v>2</v>
-      </c>
-      <c r="G17" t="s">
-        <v>43</v>
-      </c>
-      <c r="H17" s="7">
+      <c r="H17" s="3">
         <v>8.6999999999999993</v>
       </c>
-      <c r="I17" s="8">
+      <c r="I17" s="4">
         <v>0.7</v>
       </c>
-      <c r="J17" s="7">
+      <c r="J17" s="3">
         <v>8</v>
       </c>
-      <c r="K17" s="7">
+      <c r="K17" s="3">
         <v>715</v>
       </c>
-      <c r="L17" s="7">
+      <c r="L17" s="3">
         <v>288.7</v>
       </c>
-      <c r="M17" s="7">
+      <c r="M17" s="3">
         <v>52.7</v>
       </c>
-      <c r="N17" s="8">
-        <v>0</v>
-      </c>
-      <c r="O17" s="7">
+      <c r="N17" s="4">
+        <v>0</v>
+      </c>
+      <c r="O17" s="3">
         <v>25.09</v>
       </c>
-      <c r="P17" s="7">
+      <c r="P17" s="3">
         <v>0.46</v>
       </c>
-      <c r="Q17" s="8">
+      <c r="Q17" s="4">
         <v>0.185</v>
       </c>
-      <c r="R17" s="7">
+      <c r="R17" s="3">
         <v>0.54</v>
       </c>
-      <c r="S17" s="8">
-        <v>0</v>
-      </c>
-      <c r="T17" s="7">
+      <c r="S17" s="4">
+        <v>0</v>
+      </c>
+      <c r="T17" s="3">
         <v>277.89999999999998</v>
       </c>
-      <c r="U17" s="7">
+      <c r="U17" s="3">
         <v>1.36</v>
       </c>
-      <c r="V17" s="7">
+      <c r="V17" s="3">
         <v>16.100000000000001</v>
       </c>
       <c r="W17" s="2">
         <v>0</v>
       </c>
-      <c r="X17" s="7"/>
-    </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X17" s="3"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>254952</v>
       </c>
       <c r="B18" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C18" t="s">
+        <v>37</v>
+      </c>
+      <c r="D18" t="s">
         <v>38</v>
       </c>
-      <c r="D18" t="s">
-        <v>39</v>
-      </c>
       <c r="E18">
         <v>2</v>
       </c>
       <c r="F18">
         <v>2</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="3">
         <v>6.6999999999999993</v>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="3">
         <v>4.0999999999999996</v>
       </c>
-      <c r="J18" s="7">
+      <c r="J18" s="3">
         <v>2.6</v>
       </c>
-      <c r="K18" s="7">
+      <c r="K18" s="3">
         <v>267</v>
       </c>
-      <c r="L18" s="7">
+      <c r="L18" s="3">
         <v>424.5</v>
       </c>
-      <c r="M18" s="7">
+      <c r="M18" s="3">
         <v>29.8</v>
       </c>
-      <c r="N18" s="8">
-        <v>0</v>
-      </c>
-      <c r="O18" s="7">
+      <c r="N18" s="4">
+        <v>0</v>
+      </c>
+      <c r="O18" s="3">
         <v>568.02</v>
       </c>
-      <c r="P18" s="7">
+      <c r="P18" s="3">
         <v>2.1</v>
       </c>
-      <c r="Q18" s="7">
+      <c r="Q18" s="3">
         <v>0.82399999999999995</v>
       </c>
-      <c r="R18" s="7">
+      <c r="R18" s="3">
         <v>1.19</v>
       </c>
-      <c r="S18" s="7">
+      <c r="S18" s="3">
         <v>0.23</v>
       </c>
-      <c r="T18" s="7">
+      <c r="T18" s="3">
         <v>355.6</v>
       </c>
-      <c r="U18" s="7">
+      <c r="U18" s="3">
         <v>3.8519999999999999</v>
       </c>
-      <c r="V18" s="7">
+      <c r="V18" s="3">
         <v>361.7</v>
       </c>
       <c r="W18" s="2">
         <v>0</v>
       </c>
-      <c r="X18" s="7"/>
-    </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X18" s="3"/>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>254953</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
+        <v>37</v>
+      </c>
+      <c r="D19" t="s">
         <v>38</v>
       </c>
-      <c r="D19" t="s">
-        <v>39</v>
-      </c>
       <c r="E19">
         <v>2</v>
       </c>
       <c r="F19">
         <v>2</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="3">
         <v>16.2</v>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="3">
         <v>3</v>
       </c>
-      <c r="J19" s="7">
+      <c r="J19" s="3">
         <v>13.2</v>
       </c>
-      <c r="K19" s="7">
+      <c r="K19" s="3">
         <v>705</v>
       </c>
-      <c r="L19" s="7">
+      <c r="L19" s="3">
         <v>853.7</v>
       </c>
-      <c r="M19" s="7">
+      <c r="M19" s="3">
         <v>24.8</v>
       </c>
-      <c r="N19" s="8">
-        <v>0</v>
-      </c>
-      <c r="O19" s="7">
+      <c r="N19" s="4">
+        <v>0</v>
+      </c>
+      <c r="O19" s="3">
         <v>62.17</v>
       </c>
-      <c r="P19" s="7">
+      <c r="P19" s="3">
         <v>6.02</v>
       </c>
-      <c r="Q19" s="7">
+      <c r="Q19" s="3">
         <v>4.8760000000000003</v>
       </c>
-      <c r="R19" s="7">
+      <c r="R19" s="3">
         <v>2.56</v>
       </c>
-      <c r="S19" s="7">
+      <c r="S19" s="3">
         <v>0.24</v>
       </c>
-      <c r="T19" s="7">
+      <c r="T19" s="3">
         <v>214</v>
       </c>
-      <c r="U19" s="7">
+      <c r="U19" s="3">
         <v>2.6539999999999999</v>
       </c>
-      <c r="V19" s="7">
+      <c r="V19" s="3">
         <v>62.9</v>
       </c>
       <c r="W19" s="2">
         <v>2.5999999999999999E-2</v>
       </c>
-      <c r="X19" s="7"/>
-    </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X19" s="3"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>254954</v>
       </c>
       <c r="B20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C20" t="s">
+        <v>37</v>
+      </c>
+      <c r="D20" t="s">
         <v>38</v>
       </c>
-      <c r="D20" t="s">
-        <v>39</v>
-      </c>
       <c r="E20">
         <v>2</v>
       </c>
       <c r="F20">
         <v>2</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="3">
         <v>20.5</v>
       </c>
-      <c r="I20" s="8">
+      <c r="I20" s="4">
         <v>1.9</v>
       </c>
-      <c r="J20" s="7">
+      <c r="J20" s="3">
         <v>18.600000000000001</v>
       </c>
-      <c r="K20" s="7">
+      <c r="K20" s="3">
         <v>400</v>
       </c>
-      <c r="L20" s="7">
+      <c r="L20" s="3">
         <v>424.8</v>
       </c>
-      <c r="M20" s="7">
+      <c r="M20" s="3">
         <v>113</v>
       </c>
-      <c r="N20" s="8">
-        <v>0</v>
-      </c>
-      <c r="O20" s="7">
+      <c r="N20" s="4">
+        <v>0</v>
+      </c>
+      <c r="O20" s="3">
         <v>458.44</v>
       </c>
-      <c r="P20" s="7">
+      <c r="P20" s="3">
         <v>3.24</v>
       </c>
-      <c r="Q20" s="7">
+      <c r="Q20" s="3">
         <v>0.92400000000000004</v>
       </c>
-      <c r="R20" s="7">
+      <c r="R20" s="3">
         <v>2.88</v>
       </c>
-      <c r="S20" s="8">
+      <c r="S20" s="4">
         <v>0.18</v>
       </c>
-      <c r="T20" s="7">
+      <c r="T20" s="3">
         <v>228.7</v>
       </c>
-      <c r="U20" s="7">
+      <c r="U20" s="3">
         <v>4.3159999999999998</v>
       </c>
-      <c r="V20" s="7">
+      <c r="V20" s="3">
         <v>449.8</v>
       </c>
       <c r="W20" s="2">
         <v>0</v>
       </c>
-      <c r="X20" s="7"/>
-    </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X20" s="3"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>254955</v>
       </c>
       <c r="B21" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" t="s">
+        <v>37</v>
+      </c>
+      <c r="D21" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21">
+        <v>2</v>
+      </c>
+      <c r="F21">
+        <v>2</v>
+      </c>
+      <c r="G21" t="s">
         <v>47</v>
       </c>
-      <c r="C21" t="s">
-        <v>38</v>
-      </c>
-      <c r="D21" t="s">
-        <v>39</v>
-      </c>
-      <c r="E21">
-        <v>2</v>
-      </c>
-      <c r="F21">
-        <v>2</v>
-      </c>
-      <c r="G21" t="s">
-        <v>48</v>
-      </c>
-      <c r="H21" s="7">
+      <c r="H21" s="3">
         <v>29.5</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J21" s="7">
+      <c r="J21" s="3">
         <v>27.3</v>
       </c>
-      <c r="K21" s="7">
+      <c r="K21" s="3">
         <v>231</v>
       </c>
-      <c r="L21" s="7">
+      <c r="L21" s="3">
         <v>230.5</v>
       </c>
-      <c r="M21" s="7">
+      <c r="M21" s="3">
         <v>96.2</v>
       </c>
-      <c r="N21" s="7">
+      <c r="N21" s="3">
         <v>0.28000000000000003</v>
       </c>
-      <c r="O21" s="7">
+      <c r="O21" s="3">
         <v>320.44</v>
       </c>
-      <c r="P21" s="7">
+      <c r="P21" s="3">
         <v>3.21</v>
       </c>
-      <c r="Q21" s="7">
+      <c r="Q21" s="3">
         <v>1.214</v>
       </c>
-      <c r="R21" s="7">
+      <c r="R21" s="3">
         <v>1.71</v>
       </c>
-      <c r="S21" s="7">
+      <c r="S21" s="3">
         <v>0.48</v>
       </c>
-      <c r="T21" s="7">
+      <c r="T21" s="3">
         <v>248.9</v>
       </c>
-      <c r="U21" s="7">
+      <c r="U21" s="3">
         <v>5.1239999999999997</v>
       </c>
-      <c r="V21" s="7">
+      <c r="V21" s="3">
         <v>200.4</v>
       </c>
       <c r="W21" s="2">
         <v>0.157</v>
       </c>
-      <c r="X21" s="7"/>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X21" s="3"/>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>254956</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C22" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" t="s">
         <v>38</v>
       </c>
-      <c r="D22" t="s">
-        <v>39</v>
-      </c>
       <c r="E22">
         <v>2</v>
       </c>
       <c r="F22">
         <v>2</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="3">
         <v>9.2000000000000011</v>
       </c>
-      <c r="I22" s="8">
+      <c r="I22" s="4">
         <v>1.3</v>
       </c>
-      <c r="J22" s="7">
+      <c r="J22" s="3">
         <v>7.9</v>
       </c>
-      <c r="K22" s="7">
+      <c r="K22" s="3">
         <v>107</v>
       </c>
-      <c r="L22" s="7">
+      <c r="L22" s="3">
         <v>170.2</v>
       </c>
-      <c r="M22" s="7">
+      <c r="M22" s="3">
         <v>49.9</v>
       </c>
-      <c r="N22" s="8">
-        <v>0</v>
-      </c>
-      <c r="O22" s="7">
+      <c r="N22" s="4">
+        <v>0</v>
+      </c>
+      <c r="O22" s="3">
         <v>69.33</v>
       </c>
-      <c r="P22" s="7">
+      <c r="P22" s="3">
         <v>0.37</v>
       </c>
-      <c r="Q22" s="7">
+      <c r="Q22" s="3">
         <v>0.24399999999999999</v>
       </c>
-      <c r="R22" s="7">
+      <c r="R22" s="3">
         <v>0.24</v>
       </c>
-      <c r="S22" s="8">
-        <v>0</v>
-      </c>
-      <c r="T22" s="7">
+      <c r="S22" s="4">
+        <v>0</v>
+      </c>
+      <c r="T22" s="3">
         <v>106.4</v>
       </c>
-      <c r="U22" s="7">
+      <c r="U22" s="3">
         <v>1.9079999999999999</v>
       </c>
-      <c r="V22" s="7">
+      <c r="V22" s="3">
         <v>21.6</v>
       </c>
       <c r="W22" s="2">
         <v>6.0999999999999999E-2</v>
       </c>
-      <c r="X22" s="7"/>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X22" s="3"/>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>254957</v>
       </c>
       <c r="B23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C23" t="s">
+        <v>37</v>
+      </c>
+      <c r="D23" t="s">
         <v>38</v>
       </c>
-      <c r="D23" t="s">
-        <v>39</v>
-      </c>
       <c r="E23">
         <v>2</v>
       </c>
       <c r="F23">
         <v>2</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="3">
         <v>10.1</v>
       </c>
-      <c r="I23" s="8">
+      <c r="I23" s="4">
         <v>0.8</v>
       </c>
-      <c r="J23" s="7">
+      <c r="J23" s="3">
         <v>9.3000000000000007</v>
       </c>
-      <c r="K23" s="7">
+      <c r="K23" s="3">
         <v>799</v>
       </c>
-      <c r="L23" s="7">
+      <c r="L23" s="3">
         <v>647.9</v>
       </c>
-      <c r="M23" s="7">
+      <c r="M23" s="3">
         <v>23.2</v>
       </c>
-      <c r="N23" s="8">
-        <v>0</v>
-      </c>
-      <c r="O23" s="7">
+      <c r="N23" s="4">
+        <v>0</v>
+      </c>
+      <c r="O23" s="3">
         <v>56.9</v>
       </c>
-      <c r="P23" s="7">
+      <c r="P23" s="3">
         <v>0.84</v>
       </c>
-      <c r="Q23" s="8">
+      <c r="Q23" s="4">
         <v>0.17</v>
       </c>
-      <c r="R23" s="7">
+      <c r="R23" s="3">
         <v>0.49</v>
       </c>
-      <c r="S23" s="8">
+      <c r="S23" s="4">
         <v>0.04</v>
       </c>
-      <c r="T23" s="7">
+      <c r="T23" s="3">
         <v>131.19999999999999</v>
       </c>
-      <c r="U23" s="7">
+      <c r="U23" s="3">
         <v>2.2679999999999998</v>
       </c>
-      <c r="V23" s="7">
+      <c r="V23" s="3">
         <v>30.8</v>
       </c>
       <c r="W23" s="2">
         <v>9.9000000000000005E-2</v>
       </c>
-      <c r="X23" s="7"/>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X23" s="3"/>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>254958</v>
       </c>
       <c r="B24" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C24" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" t="s">
         <v>38</v>
       </c>
-      <c r="D24" t="s">
-        <v>39</v>
-      </c>
       <c r="E24">
         <v>2</v>
       </c>
       <c r="F24">
         <v>2</v>
       </c>
-      <c r="H24" s="7">
+      <c r="H24" s="3">
         <v>14.5</v>
       </c>
-      <c r="I24" s="8">
+      <c r="I24" s="4">
         <v>0.9</v>
       </c>
-      <c r="J24" s="7">
+      <c r="J24" s="3">
         <v>13.6</v>
       </c>
-      <c r="K24" s="7">
+      <c r="K24" s="3">
         <v>1053</v>
       </c>
-      <c r="L24" s="7">
+      <c r="L24" s="3">
         <v>453.5</v>
       </c>
-      <c r="M24" s="7">
+      <c r="M24" s="3">
         <v>49</v>
       </c>
-      <c r="N24" s="8">
-        <v>0</v>
-      </c>
-      <c r="O24" s="7">
+      <c r="N24" s="4">
+        <v>0</v>
+      </c>
+      <c r="O24" s="3">
         <v>33.770000000000003</v>
       </c>
-      <c r="P24" s="7">
+      <c r="P24" s="3">
         <v>1.05</v>
       </c>
-      <c r="Q24" s="7">
+      <c r="Q24" s="3">
         <v>0.52</v>
       </c>
-      <c r="R24" s="7">
+      <c r="R24" s="3">
         <v>0.63</v>
       </c>
-      <c r="S24" s="7">
+      <c r="S24" s="3">
         <v>0.49</v>
       </c>
-      <c r="T24" s="7">
+      <c r="T24" s="3">
         <v>237.8</v>
       </c>
-      <c r="U24" s="7">
+      <c r="U24" s="3">
         <v>2.4540000000000002</v>
       </c>
-      <c r="V24" s="7">
+      <c r="V24" s="3">
         <v>33.5</v>
       </c>
       <c r="W24" s="2">
         <v>0</v>
       </c>
-      <c r="X24" s="7"/>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X24" s="3"/>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>254959</v>
       </c>
       <c r="B25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C25" t="s">
+        <v>37</v>
+      </c>
+      <c r="D25" t="s">
         <v>38</v>
       </c>
-      <c r="D25" t="s">
-        <v>39</v>
-      </c>
       <c r="E25">
         <v>2</v>
       </c>
       <c r="F25">
         <v>2</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="3">
         <v>7.5</v>
       </c>
-      <c r="I25" s="8">
+      <c r="I25" s="4">
         <v>1.4</v>
       </c>
-      <c r="J25" s="7">
+      <c r="J25" s="3">
         <v>6.1</v>
       </c>
-      <c r="K25" s="7">
+      <c r="K25" s="3">
         <v>747</v>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="3">
         <v>612.20000000000005</v>
       </c>
-      <c r="M25" s="7">
+      <c r="M25" s="3">
         <v>102</v>
       </c>
-      <c r="N25" s="8">
+      <c r="N25" s="4">
         <v>0.08</v>
       </c>
-      <c r="O25" s="7">
+      <c r="O25" s="3">
         <v>4.87</v>
       </c>
-      <c r="P25" s="7">
+      <c r="P25" s="3">
         <v>2.08</v>
       </c>
-      <c r="Q25" s="7">
+      <c r="Q25" s="3">
         <v>0.375</v>
       </c>
-      <c r="R25" s="7">
+      <c r="R25" s="3">
         <v>1.99</v>
       </c>
-      <c r="S25" s="8">
-        <v>0</v>
-      </c>
-      <c r="T25" s="7">
+      <c r="S25" s="4">
+        <v>0</v>
+      </c>
+      <c r="T25" s="3">
         <v>83.4</v>
       </c>
-      <c r="U25" s="7">
+      <c r="U25" s="3">
         <v>10.471</v>
       </c>
-      <c r="V25" s="7">
+      <c r="V25" s="3">
         <v>13.9</v>
       </c>
       <c r="W25" s="2">
         <v>0.05</v>
       </c>
-      <c r="X25" s="7"/>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X25" s="3"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>254960</v>
       </c>
       <c r="B26" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" t="s">
         <v>53</v>
       </c>
-      <c r="C26" t="s">
-        <v>54</v>
-      </c>
       <c r="D26" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E26">
         <v>2</v>
@@ -2104,68 +2114,68 @@
       <c r="F26">
         <v>2</v>
       </c>
-      <c r="H26" s="7">
+      <c r="H26" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="I26" s="8">
+      <c r="I26" s="4">
         <v>0.9</v>
       </c>
-      <c r="J26" s="8">
+      <c r="J26" s="4">
         <v>1.3</v>
       </c>
-      <c r="K26" s="7">
+      <c r="K26" s="3">
         <v>351</v>
       </c>
-      <c r="L26" s="7">
+      <c r="L26" s="3">
         <v>164.9</v>
       </c>
-      <c r="M26" s="7">
+      <c r="M26" s="3">
         <v>4.9000000000000004</v>
       </c>
-      <c r="N26" s="8">
-        <v>0</v>
-      </c>
-      <c r="O26" s="7">
+      <c r="N26" s="4">
+        <v>0</v>
+      </c>
+      <c r="O26" s="3">
         <v>733.06</v>
       </c>
-      <c r="P26" s="7">
+      <c r="P26" s="3">
         <v>0.53</v>
       </c>
-      <c r="Q26" s="7">
+      <c r="Q26" s="3">
         <v>0.25</v>
       </c>
-      <c r="R26" s="7">
+      <c r="R26" s="3">
         <v>0.38</v>
       </c>
-      <c r="S26" s="8">
+      <c r="S26" s="4">
         <v>0.08</v>
       </c>
-      <c r="T26" s="7">
+      <c r="T26" s="3">
         <v>46.3</v>
       </c>
-      <c r="U26" s="7">
+      <c r="U26" s="3">
         <v>2.1480000000000001</v>
       </c>
-      <c r="V26" s="7">
+      <c r="V26" s="3">
         <v>768.7</v>
       </c>
       <c r="W26">
         <v>0.25700000000000001</v>
       </c>
-      <c r="X26" s="7"/>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X26" s="3"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>254961</v>
       </c>
       <c r="B27" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C27" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E27">
         <v>2</v>
@@ -2173,68 +2183,68 @@
       <c r="F27">
         <v>2</v>
       </c>
-      <c r="H27" s="7">
+      <c r="H27" s="3">
         <v>6</v>
       </c>
-      <c r="I27" s="8">
+      <c r="I27" s="4">
         <v>0.9</v>
       </c>
-      <c r="J27" s="7">
+      <c r="J27" s="3">
         <v>5.0999999999999996</v>
       </c>
-      <c r="K27" s="7">
+      <c r="K27" s="3">
         <v>113</v>
       </c>
-      <c r="L27" s="7">
+      <c r="L27" s="3">
         <v>262.2</v>
       </c>
-      <c r="M27" s="7">
+      <c r="M27" s="3">
         <v>12.1</v>
       </c>
-      <c r="N27" s="8">
-        <v>0</v>
-      </c>
-      <c r="O27" s="7">
+      <c r="N27" s="4">
+        <v>0</v>
+      </c>
+      <c r="O27" s="3">
         <v>557.96</v>
       </c>
-      <c r="P27" s="7">
+      <c r="P27" s="3">
         <v>0.77</v>
       </c>
-      <c r="Q27" s="7">
+      <c r="Q27" s="3">
         <v>0.21199999999999999</v>
       </c>
-      <c r="R27" s="7">
+      <c r="R27" s="3">
         <v>0.4</v>
       </c>
-      <c r="S27" s="8">
+      <c r="S27" s="4">
         <v>0.01</v>
       </c>
-      <c r="T27" s="7">
+      <c r="T27" s="3">
         <v>72.5</v>
       </c>
-      <c r="U27" s="7">
+      <c r="U27" s="3">
         <v>1.9279999999999999</v>
       </c>
-      <c r="V27" s="7">
+      <c r="V27" s="3">
         <v>443.2</v>
       </c>
       <c r="W27" s="2">
         <v>6.7000000000000004E-2</v>
       </c>
-      <c r="X27" s="7"/>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X27" s="3"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>254962</v>
       </c>
       <c r="B28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E28">
         <v>2</v>
@@ -2242,68 +2252,68 @@
       <c r="F28">
         <v>2</v>
       </c>
-      <c r="H28" s="7">
+      <c r="H28" s="3">
         <v>3.9</v>
       </c>
-      <c r="I28" s="8">
+      <c r="I28" s="4">
         <v>1.7</v>
       </c>
-      <c r="J28" s="7">
+      <c r="J28" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="K28" s="7">
+      <c r="K28" s="3">
         <v>247</v>
       </c>
-      <c r="L28" s="7">
+      <c r="L28" s="3">
         <v>221.3</v>
       </c>
-      <c r="M28" s="7">
+      <c r="M28" s="3">
         <v>16.600000000000001</v>
       </c>
-      <c r="N28" s="7">
+      <c r="N28" s="3">
         <v>0.42</v>
       </c>
-      <c r="O28" s="7">
+      <c r="O28" s="3">
         <v>503.54</v>
       </c>
-      <c r="P28" s="7">
+      <c r="P28" s="3">
         <v>0.94</v>
       </c>
-      <c r="Q28" s="8">
+      <c r="Q28" s="4">
         <v>0.182</v>
       </c>
-      <c r="R28" s="7">
+      <c r="R28" s="3">
         <v>0.41</v>
       </c>
-      <c r="S28" s="7">
+      <c r="S28" s="3">
         <v>0.22</v>
       </c>
-      <c r="T28" s="7">
+      <c r="T28" s="3">
         <v>157.9</v>
       </c>
-      <c r="U28" s="7">
+      <c r="U28" s="3">
         <v>2.3359999999999999</v>
       </c>
-      <c r="V28" s="7">
+      <c r="V28" s="3">
         <v>389.3</v>
       </c>
       <c r="W28" s="2">
         <v>0</v>
       </c>
-      <c r="X28" s="7"/>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X28" s="3"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>254963</v>
       </c>
       <c r="B29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E29">
         <v>2</v>
@@ -2311,68 +2321,68 @@
       <c r="F29">
         <v>2</v>
       </c>
-      <c r="H29" s="8">
+      <c r="H29" s="4">
         <v>1.3</v>
       </c>
-      <c r="I29" s="8">
+      <c r="I29" s="4">
         <v>1</v>
       </c>
-      <c r="J29" s="8">
+      <c r="J29" s="4">
         <v>0.3</v>
       </c>
-      <c r="K29" s="7">
+      <c r="K29" s="3">
         <v>182</v>
       </c>
-      <c r="L29" s="7">
+      <c r="L29" s="3">
         <v>180</v>
       </c>
-      <c r="M29" s="7">
+      <c r="M29" s="3">
         <v>10</v>
       </c>
-      <c r="N29" s="8">
-        <v>0</v>
-      </c>
-      <c r="O29" s="7">
+      <c r="N29" s="4">
+        <v>0</v>
+      </c>
+      <c r="O29" s="3">
         <v>1734.33</v>
       </c>
-      <c r="P29" s="7">
+      <c r="P29" s="3">
         <v>4.9400000000000004</v>
       </c>
-      <c r="Q29" s="7">
+      <c r="Q29" s="3">
         <v>0.22</v>
       </c>
-      <c r="R29" s="7">
+      <c r="R29" s="3">
         <v>0.77</v>
       </c>
-      <c r="S29" s="8">
+      <c r="S29" s="4">
         <v>0.16</v>
       </c>
-      <c r="T29" s="7">
+      <c r="T29" s="3">
         <v>136.1</v>
       </c>
-      <c r="U29" s="7">
+      <c r="U29" s="3">
         <v>2.7770000000000001</v>
       </c>
-      <c r="V29" s="7">
+      <c r="V29" s="3">
         <v>542.29999999999995</v>
       </c>
       <c r="W29" s="2">
         <v>0.13100000000000001</v>
       </c>
-      <c r="X29" s="7"/>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X29" s="3"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A30">
         <v>254964</v>
       </c>
       <c r="B30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E30">
         <v>2</v>
@@ -2380,68 +2390,68 @@
       <c r="F30">
         <v>2</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="3">
         <v>2.6</v>
       </c>
-      <c r="I30" s="8">
+      <c r="I30" s="4">
         <v>1.3</v>
       </c>
-      <c r="J30" s="8">
+      <c r="J30" s="4">
         <v>1.3</v>
       </c>
-      <c r="K30" s="7">
+      <c r="K30" s="3">
         <v>178</v>
       </c>
-      <c r="L30" s="7">
+      <c r="L30" s="3">
         <v>201.9</v>
       </c>
-      <c r="M30" s="7">
+      <c r="M30" s="3">
         <v>13.5</v>
       </c>
-      <c r="N30" s="8">
-        <v>0</v>
-      </c>
-      <c r="O30" s="7">
+      <c r="N30" s="4">
+        <v>0</v>
+      </c>
+      <c r="O30" s="3">
         <v>1709.69</v>
       </c>
-      <c r="P30" s="7">
+      <c r="P30" s="3">
         <v>0.96</v>
       </c>
-      <c r="Q30" s="7">
+      <c r="Q30" s="3">
         <v>0.23200000000000001</v>
       </c>
-      <c r="R30" s="7">
+      <c r="R30" s="3">
         <v>0.22</v>
       </c>
-      <c r="S30" s="7">
+      <c r="S30" s="3">
         <v>0.21</v>
       </c>
-      <c r="T30" s="7">
+      <c r="T30" s="3">
         <v>118.3</v>
       </c>
-      <c r="U30" s="7">
+      <c r="U30" s="3">
         <v>3.5880000000000001</v>
       </c>
-      <c r="V30" s="7">
+      <c r="V30" s="3">
         <v>445.1</v>
       </c>
       <c r="W30" s="2">
         <v>0.14799999999999999</v>
       </c>
-      <c r="X30" s="7"/>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.4">
+      <c r="X30" s="3"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.45">
       <c r="A31">
         <v>254965</v>
       </c>
       <c r="B31" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C31" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E31">
         <v>2</v>
@@ -2449,55 +2459,55 @@
       <c r="F31">
         <v>2</v>
       </c>
-      <c r="H31" s="7">
+      <c r="H31" s="3">
         <v>20.2</v>
       </c>
-      <c r="I31" s="8">
+      <c r="I31" s="4">
         <v>1.2</v>
       </c>
-      <c r="J31" s="7">
+      <c r="J31" s="3">
         <v>19</v>
       </c>
-      <c r="K31" s="7">
+      <c r="K31" s="3">
         <v>179</v>
       </c>
-      <c r="L31" s="7">
+      <c r="L31" s="3">
         <v>289.39999999999998</v>
       </c>
-      <c r="M31" s="7">
+      <c r="M31" s="3">
         <v>59.5</v>
       </c>
-      <c r="N31" s="8">
+      <c r="N31" s="4">
         <v>0.14000000000000001</v>
       </c>
-      <c r="O31" s="7">
+      <c r="O31" s="3">
         <v>1305.3800000000001</v>
       </c>
-      <c r="P31" s="7">
+      <c r="P31" s="3">
         <v>2.99</v>
       </c>
-      <c r="Q31" s="7">
+      <c r="Q31" s="3">
         <v>0.40600000000000003</v>
       </c>
-      <c r="R31" s="7">
+      <c r="R31" s="3">
         <v>2.0699999999999998</v>
       </c>
-      <c r="S31" s="7">
+      <c r="S31" s="3">
         <v>0.68</v>
       </c>
-      <c r="T31" s="7">
+      <c r="T31" s="3">
         <v>108.9</v>
       </c>
-      <c r="U31" s="7">
+      <c r="U31" s="3">
         <v>2.7029999999999998</v>
       </c>
-      <c r="V31" s="7">
+      <c r="V31" s="3">
         <v>430.8</v>
       </c>
       <c r="W31" s="2">
         <v>0.127</v>
       </c>
-      <c r="X31" s="7"/>
+      <c r="X31" s="3"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
@@ -2509,6 +2519,7 @@
     <mergeCell ref="A4:W4"/>
     <mergeCell ref="A5:W5"/>
   </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>